<commit_message>
Update critical elevations in Powell and Mead
</commit_message>
<xml_diff>
--- a/R-Figs/AutoReadUSBRData/Bathymetry.xlsx
+++ b/R-Figs/AutoReadUSBRData/Bathymetry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2558001745240/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516BF7B1-2E6E-4F66-A02E-D0567C567724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{516BF7B1-2E6E-4F66-A02E-D0567C567724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E45572-31A6-463B-9E3E-18C33568AD0B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>Elevation (ft)</t>
   </si>
@@ -141,6 +141,18 @@
   </si>
   <si>
     <t>Volume above 3,514</t>
+  </si>
+  <si>
+    <t>Volume above 3490</t>
+  </si>
+  <si>
+    <t>Mead Elevation</t>
+  </si>
+  <si>
+    <t>Volume above 1000</t>
+  </si>
+  <si>
+    <t>Volume above 950</t>
   </si>
 </sst>
 </file>
@@ -328,7 +340,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -429,6 +441,9 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9360,7 +9375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
@@ -9432,6 +9447,9 @@
       <c r="K11" s="39" t="s">
         <v>28</v>
       </c>
+      <c r="L11" s="40" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="35" t="s">
@@ -9463,6 +9481,10 @@
         <f t="shared" ref="K12:K15" si="0">I12-I$16</f>
         <v>1.8358071300000018</v>
       </c>
+      <c r="L12" s="38">
+        <f>I12-I$19</f>
+        <v>3.0260774310000018</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="35" t="s">
@@ -9495,8 +9517,8 @@
         <v>1.2054862920000007</v>
       </c>
       <c r="L13" s="38">
-        <f>I13-I14</f>
-        <v>0.41931773800000016</v>
+        <f t="shared" ref="L13:L19" si="1">I13-I$19</f>
+        <v>2.3957565930000007</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -9515,6 +9537,10 @@
         <f t="shared" si="0"/>
         <v>0.78616855400000052</v>
       </c>
+      <c r="L14" s="38">
+        <f t="shared" si="1"/>
+        <v>1.9764388550000005</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G15">
@@ -9532,6 +9558,10 @@
         <f t="shared" si="0"/>
         <v>0.61193845800000091</v>
       </c>
+      <c r="L15" s="38">
+        <f t="shared" si="1"/>
+        <v>1.8022087590000009</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G16">
@@ -9549,8 +9579,12 @@
         <f>I16-I$16</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="7:9" x14ac:dyDescent="0.35">
+      <c r="L16" s="38">
+        <f t="shared" si="1"/>
+        <v>1.190270301</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G17">
         <v>3510</v>
       </c>
@@ -9562,8 +9596,12 @@
         <f>H17-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
         <v>4.7210644459999997</v>
       </c>
-    </row>
-    <row r="18" spans="7:9" x14ac:dyDescent="0.35">
+      <c r="L17" s="38">
+        <f t="shared" si="1"/>
+        <v>0.97835029600000034</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G18">
         <v>3500</v>
       </c>
@@ -9575,8 +9613,12 @@
         <f>H18-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
         <v>4.2158051219999999</v>
       </c>
-    </row>
-    <row r="19" spans="7:9" x14ac:dyDescent="0.35">
+      <c r="L18" s="38">
+        <f t="shared" si="1"/>
+        <v>0.4730909720000005</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G19">
         <v>3490</v>
       </c>
@@ -9588,6 +9630,179 @@
         <f>H19-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
         <v>3.7427141499999994</v>
       </c>
+      <c r="L19" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="G22" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="H22" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="40" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G23">
+        <v>895</v>
+      </c>
+      <c r="H23" s="37">
+        <f>VLOOKUP($G23,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>2.0350000000000001</v>
+      </c>
+      <c r="I23" s="37">
+        <f>VLOOKUP($G23,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="38">
+        <f>I23-I$26</f>
+        <v>-4.475301</v>
+      </c>
+      <c r="L23" s="38">
+        <f>I23-I$24</f>
+        <v>-2.005585</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G24">
+        <v>950</v>
+      </c>
+      <c r="H24" s="37">
+        <f>VLOOKUP($G24,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>4.0405850000000001</v>
+      </c>
+      <c r="I24" s="37">
+        <f>VLOOKUP($G24,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>2.005585</v>
+      </c>
+      <c r="K24" s="38">
+        <f t="shared" ref="K24:K28" si="2">I24-I$26</f>
+        <v>-2.469716</v>
+      </c>
+      <c r="L24" s="38">
+        <f t="shared" ref="L24:L28" si="3">I24-I$24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G25">
+        <v>975</v>
+      </c>
+      <c r="H25" s="37">
+        <f>VLOOKUP($G25,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>5.1913530000000003</v>
+      </c>
+      <c r="I25" s="37">
+        <f>VLOOKUP($G25,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>3.1563530000000002</v>
+      </c>
+      <c r="K25" s="38">
+        <f t="shared" si="2"/>
+        <v>-1.3189479999999998</v>
+      </c>
+      <c r="L25" s="38">
+        <f t="shared" si="3"/>
+        <v>1.1507680000000002</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G26">
+        <v>1000</v>
+      </c>
+      <c r="H26" s="37">
+        <f>VLOOKUP($G26,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>6.5103010000000001</v>
+      </c>
+      <c r="I26" s="37">
+        <f>VLOOKUP($G26,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>4.475301</v>
+      </c>
+      <c r="K26" s="38">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L26" s="38">
+        <f t="shared" si="3"/>
+        <v>2.469716</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G27">
+        <v>1020</v>
+      </c>
+      <c r="H27" s="37">
+        <f>VLOOKUP($G27,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>7.6995930000000001</v>
+      </c>
+      <c r="I27" s="37">
+        <f>VLOOKUP($G27,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>5.664593</v>
+      </c>
+      <c r="K27" s="38">
+        <f t="shared" si="2"/>
+        <v>1.189292</v>
+      </c>
+      <c r="L27" s="38">
+        <f t="shared" si="3"/>
+        <v>3.659008</v>
+      </c>
+    </row>
+    <row r="28" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G28">
+        <v>1040</v>
+      </c>
+      <c r="H28" s="37">
+        <f>VLOOKUP($G28,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>9.0126650000000001</v>
+      </c>
+      <c r="I28" s="37">
+        <f>VLOOKUP($G28,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>6.977665</v>
+      </c>
+      <c r="K28" s="38">
+        <f t="shared" si="2"/>
+        <v>2.502364</v>
+      </c>
+      <c r="L28" s="38">
+        <f t="shared" si="3"/>
+        <v>4.9720800000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G29">
+        <v>1041</v>
+      </c>
+      <c r="H29" s="37">
+        <f>VLOOKUP($G29,'Mead-Bathymetry'!$A$2:$C$673,3)/1000000</f>
+        <v>9.0816680000000005</v>
+      </c>
+      <c r="I29" s="37">
+        <f>VLOOKUP($G29,'Mead-Bathymetry'!$A$2:$C$673,2)/1000000</f>
+        <v>7.0466680000000004</v>
+      </c>
+      <c r="K29" s="38">
+        <f t="shared" ref="K29" si="4">I29-I$26</f>
+        <v>2.5713670000000004</v>
+      </c>
+      <c r="L29" s="38">
+        <f t="shared" ref="L29" si="5">I29-I$24</f>
+        <v>5.0410830000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="H30" s="37"/>
+      <c r="I30" s="37"/>
+      <c r="L30" s="38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>